<commit_message>
feat(tv1): finalize TV1 deliverables with test logs, killer adversary suite, and assignment status
</commit_message>
<xml_diff>
--- a/docs/Phan_cong_chuan_theo_de_Sorting_pdqsort.xlsx
+++ b/docs/Phan_cong_chuan_theo_de_Sorting_pdqsort.xlsx
@@ -1615,7 +1615,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>